<commit_message>
graphs and sensitivities for review
</commit_message>
<xml_diff>
--- a/Social charging model/SCM_export_results_behaviours.xlsx
+++ b/Social charging model/SCM_export_results_behaviours.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naudl\Documents\GitHub\social-charging-model\Social charging model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902B9DF7-F216-4A0A-B8DA-CE39AE26134B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10674DE8-6E2A-43C4-86C9-4B0EBC74DDB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{3758AFA0-8E81-488E-A41A-47B84DA45D8A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3758AFA0-8E81-488E-A41A-47B84DA45D8A}"/>
   </bookViews>
   <sheets>
     <sheet name="per_week" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
   <si>
     <t>scenario</t>
   </si>
@@ -50,15 +50,6 @@
     <t>u_lwc</t>
   </si>
   <si>
-    <t>l_oomc</t>
-  </si>
-  <si>
-    <t>m_oomc</t>
-  </si>
-  <si>
-    <t>u_oomc</t>
-  </si>
-  <si>
     <t>m_luc</t>
   </si>
   <si>
@@ -77,15 +68,6 @@
     <t>u_cs</t>
   </si>
   <si>
-    <t>m_cspd</t>
-  </si>
-  <si>
-    <t>l_cspd</t>
-  </si>
-  <si>
-    <t>u_cspd</t>
-  </si>
-  <si>
     <t>m_rcspd</t>
   </si>
   <si>
@@ -399,6 +381,48 @@
   </si>
   <si>
     <t>trips_50</t>
+  </si>
+  <si>
+    <t>randomMissFactorB2</t>
+  </si>
+  <si>
+    <t>m_oomcs</t>
+  </si>
+  <si>
+    <t>l_oomcs</t>
+  </si>
+  <si>
+    <t>u_oomcs</t>
+  </si>
+  <si>
+    <t>m_oomckWh</t>
+  </si>
+  <si>
+    <t>l_oomckWh</t>
+  </si>
+  <si>
+    <t>u_oomckWh</t>
+  </si>
+  <si>
+    <t>rechecksPerDay</t>
+  </si>
+  <si>
+    <t>m_cspw</t>
+  </si>
+  <si>
+    <t>l_cspw</t>
+  </si>
+  <si>
+    <t>u_cspw</t>
+  </si>
+  <si>
+    <t>EMASmoothingFactor</t>
+  </si>
+  <si>
+    <t>negBiasFactor</t>
+  </si>
+  <si>
+    <t>surprisalFunction</t>
   </si>
 </sst>
 </file>
@@ -776,372 +800,396 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C276F534-E875-46ED-80D0-6FDBCE465A6B}">
-  <dimension ref="A1:DQ1"/>
+  <dimension ref="A1:DY1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:121" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:129" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H1" t="s">
+        <v>121</v>
+      </c>
+      <c r="I1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" t="s">
+        <v>4</v>
+      </c>
+      <c r="M1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N1" t="s">
+        <v>6</v>
+      </c>
+      <c r="O1" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" t="s">
+        <v>8</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>9</v>
+      </c>
+      <c r="R1" t="s">
+        <v>123</v>
+      </c>
+      <c r="S1" t="s">
+        <v>124</v>
+      </c>
+      <c r="T1" t="s">
+        <v>125</v>
+      </c>
+      <c r="U1" t="s">
+        <v>10</v>
+      </c>
+      <c r="V1" t="s">
+        <v>11</v>
+      </c>
+      <c r="W1" t="s">
+        <v>12</v>
+      </c>
+      <c r="X1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AC1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" t="s">
+      <c r="AD1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AF1" t="s">
         <v>27</v>
       </c>
-      <c r="V1" t="s">
-        <v>26</v>
-      </c>
-      <c r="W1" t="s">
-        <v>25</v>
-      </c>
-      <c r="X1" t="s">
+      <c r="AG1" t="s">
         <v>28</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AH1" t="s">
         <v>29</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AI1" t="s">
         <v>30</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AJ1" t="s">
         <v>31</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AK1" t="s">
         <v>32</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AL1" t="s">
         <v>33</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AM1" t="s">
         <v>34</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AN1" t="s">
         <v>35</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AO1" t="s">
         <v>36</v>
       </c>
-      <c r="AG1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>55</v>
-      </c>
       <c r="AP1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AQ1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="AR1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="AS1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="AT1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="AU1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="AV1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="AW1" t="s">
         <v>44</v>
       </c>
       <c r="AX1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="AY1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="AZ1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="BA1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="BB1" t="s">
+        <v>40</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>41</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>42</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>53</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>54</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>55</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BK1" t="s">
         <v>59</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BL1" t="s">
         <v>60</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BM1" t="s">
         <v>61</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BN1" t="s">
         <v>62</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BO1" t="s">
         <v>63</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BP1" t="s">
         <v>64</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BQ1" t="s">
         <v>65</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BR1" t="s">
         <v>66</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BS1" t="s">
         <v>67</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BT1" t="s">
         <v>68</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BU1" t="s">
         <v>69</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BV1" t="s">
         <v>70</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BW1" t="s">
         <v>71</v>
       </c>
-      <c r="BO1" t="s">
+      <c r="BX1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BY1" t="s">
         <v>72</v>
       </c>
-      <c r="BP1" t="s">
-        <v>73</v>
-      </c>
-      <c r="BQ1" t="s">
+      <c r="BZ1" t="s">
         <v>74</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="CA1" t="s">
         <v>75</v>
       </c>
-      <c r="BS1" t="s">
+      <c r="CB1" t="s">
         <v>76</v>
       </c>
-      <c r="BT1" t="s">
+      <c r="CC1" t="s">
         <v>77</v>
       </c>
-      <c r="BU1" t="s">
+      <c r="CD1" t="s">
+        <v>78</v>
+      </c>
+      <c r="CE1" t="s">
         <v>79</v>
       </c>
-      <c r="BV1" t="s">
-        <v>78</v>
-      </c>
-      <c r="BW1" t="s">
+      <c r="CF1" t="s">
+        <v>13</v>
+      </c>
+      <c r="CG1" t="s">
+        <v>14</v>
+      </c>
+      <c r="CH1" t="s">
+        <v>15</v>
+      </c>
+      <c r="CI1" t="s">
+        <v>16</v>
+      </c>
+      <c r="CJ1" t="s">
+        <v>17</v>
+      </c>
+      <c r="CK1" t="s">
+        <v>52</v>
+      </c>
+      <c r="CL1" t="s">
+        <v>115</v>
+      </c>
+      <c r="CM1" t="s">
+        <v>126</v>
+      </c>
+      <c r="CN1" t="s">
+        <v>122</v>
+      </c>
+      <c r="CO1" t="s">
+        <v>127</v>
+      </c>
+      <c r="CP1" t="s">
+        <v>128</v>
+      </c>
+      <c r="CQ1" t="s">
         <v>80</v>
       </c>
-      <c r="BX1" t="s">
+      <c r="CR1" t="s">
         <v>81</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CS1" t="s">
         <v>82</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CT1" t="s">
         <v>83</v>
       </c>
-      <c r="CA1" t="s">
+      <c r="CU1" t="s">
         <v>84</v>
       </c>
-      <c r="CB1" t="s">
+      <c r="CV1" t="s">
         <v>85</v>
       </c>
-      <c r="CC1" t="s">
-        <v>19</v>
-      </c>
-      <c r="CD1" t="s">
-        <v>20</v>
-      </c>
-      <c r="CE1" t="s">
-        <v>21</v>
-      </c>
-      <c r="CF1" t="s">
-        <v>22</v>
-      </c>
-      <c r="CG1" t="s">
-        <v>23</v>
-      </c>
-      <c r="CH1" t="s">
-        <v>58</v>
-      </c>
-      <c r="CI1" t="s">
+      <c r="CW1" t="s">
         <v>86</v>
       </c>
-      <c r="CJ1" t="s">
+      <c r="CX1" t="s">
+        <v>94</v>
+      </c>
+      <c r="CY1" t="s">
+        <v>95</v>
+      </c>
+      <c r="CZ1" t="s">
+        <v>96</v>
+      </c>
+      <c r="DA1" t="s">
+        <v>97</v>
+      </c>
+      <c r="DB1" t="s">
+        <v>98</v>
+      </c>
+      <c r="DC1" t="s">
+        <v>99</v>
+      </c>
+      <c r="DD1" t="s">
+        <v>100</v>
+      </c>
+      <c r="DE1" t="s">
+        <v>101</v>
+      </c>
+      <c r="DF1" t="s">
+        <v>102</v>
+      </c>
+      <c r="DG1" t="s">
+        <v>103</v>
+      </c>
+      <c r="DH1" t="s">
+        <v>104</v>
+      </c>
+      <c r="DI1" t="s">
+        <v>105</v>
+      </c>
+      <c r="DJ1" t="s">
+        <v>106</v>
+      </c>
+      <c r="DK1" t="s">
+        <v>107</v>
+      </c>
+      <c r="DL1" t="s">
+        <v>108</v>
+      </c>
+      <c r="DM1" t="s">
+        <v>109</v>
+      </c>
+      <c r="DN1" t="s">
+        <v>110</v>
+      </c>
+      <c r="DO1" t="s">
+        <v>111</v>
+      </c>
+      <c r="DP1" t="s">
+        <v>112</v>
+      </c>
+      <c r="DQ1" t="s">
+        <v>113</v>
+      </c>
+      <c r="DR1" t="s">
+        <v>114</v>
+      </c>
+      <c r="DS1" t="s">
         <v>87</v>
       </c>
-      <c r="CK1" t="s">
+      <c r="DT1" t="s">
         <v>88</v>
       </c>
-      <c r="CL1" t="s">
+      <c r="DU1" t="s">
         <v>89</v>
       </c>
-      <c r="CM1" t="s">
+      <c r="DV1" t="s">
         <v>90</v>
       </c>
-      <c r="CN1" t="s">
+      <c r="DW1" t="s">
         <v>91</v>
       </c>
-      <c r="CO1" t="s">
+      <c r="DX1" t="s">
         <v>92</v>
       </c>
-      <c r="CP1" t="s">
-        <v>100</v>
-      </c>
-      <c r="CQ1" t="s">
-        <v>101</v>
-      </c>
-      <c r="CR1" t="s">
-        <v>102</v>
-      </c>
-      <c r="CS1" t="s">
-        <v>103</v>
-      </c>
-      <c r="CT1" t="s">
-        <v>104</v>
-      </c>
-      <c r="CU1" t="s">
-        <v>105</v>
-      </c>
-      <c r="CV1" t="s">
-        <v>106</v>
-      </c>
-      <c r="CW1" t="s">
-        <v>107</v>
-      </c>
-      <c r="CX1" t="s">
-        <v>108</v>
-      </c>
-      <c r="CY1" t="s">
-        <v>109</v>
-      </c>
-      <c r="CZ1" t="s">
-        <v>110</v>
-      </c>
-      <c r="DA1" t="s">
-        <v>111</v>
-      </c>
-      <c r="DB1" t="s">
-        <v>112</v>
-      </c>
-      <c r="DC1" t="s">
-        <v>113</v>
-      </c>
-      <c r="DD1" t="s">
-        <v>114</v>
-      </c>
-      <c r="DE1" t="s">
-        <v>115</v>
-      </c>
-      <c r="DF1" t="s">
-        <v>116</v>
-      </c>
-      <c r="DG1" t="s">
-        <v>117</v>
-      </c>
-      <c r="DH1" t="s">
-        <v>118</v>
-      </c>
-      <c r="DI1" t="s">
-        <v>119</v>
-      </c>
-      <c r="DJ1" t="s">
-        <v>120</v>
-      </c>
-      <c r="DK1" t="s">
+      <c r="DY1" t="s">
         <v>93</v>
-      </c>
-      <c r="DL1" t="s">
-        <v>94</v>
-      </c>
-      <c r="DM1" t="s">
-        <v>95</v>
-      </c>
-      <c r="DN1" t="s">
-        <v>96</v>
-      </c>
-      <c r="DO1" t="s">
-        <v>97</v>
-      </c>
-      <c r="DP1" t="s">
-        <v>98</v>
-      </c>
-      <c r="DQ1" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>